<commit_message>
correction des schemas MCD
</commit_message>
<xml_diff>
--- a/Epreuve E6/dictionnaire_de_donnee.xlsx
+++ b/Epreuve E6/dictionnaire_de_donnee.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ericn\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ericn\Desktop\M2I_Site_Web\Epreuve E6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF25136-9432-4BD2-AD0F-7A482FE6749A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6693FBFA-92C0-4CDA-A08B-DBF404314AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="11512" xr2:uid="{98FF39A9-B756-4F1B-9555-C74E8F4C24B7}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{98FF39A9-B756-4F1B-9555-C74E8F4C24B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="85">
   <si>
     <t>Données</t>
   </si>
@@ -167,12 +167,6 @@
     <t>identifiant de la réservation de l'adherent</t>
   </si>
   <si>
-    <t>ballon</t>
-  </si>
-  <si>
-    <t>id_ballon</t>
-  </si>
-  <si>
     <t>stock_base</t>
   </si>
   <si>
@@ -185,27 +179,12 @@
     <t>stock actuel de ballon</t>
   </si>
   <si>
-    <t>chasuble</t>
-  </si>
-  <si>
-    <t>id_chasuble</t>
-  </si>
-  <si>
-    <t>id d'un stock de chasuble apparatenant à un terrain d'un club</t>
-  </si>
-  <si>
     <t>id d'un stock de ballons apparatenant à un terrain d'un club</t>
   </si>
   <si>
-    <t>id_crampon</t>
-  </si>
-  <si>
     <t>id d'un stock de crampon apparatenant à un terrain d'un club</t>
   </si>
   <si>
-    <t>crampon</t>
-  </si>
-  <si>
     <t>club</t>
   </si>
   <si>
@@ -303,6 +282,15 @@
   </si>
   <si>
     <t>nombre de défaites d'un adherent sur l'ensemble de ses matchs</t>
+  </si>
+  <si>
+    <t>id_equipements</t>
+  </si>
+  <si>
+    <t>equipement</t>
+  </si>
+  <si>
+    <t>nom de l'équipement - [ballon/chasuble/crampon]</t>
   </si>
 </sst>
 </file>
@@ -357,7 +345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -368,9 +356,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5DBF5CA-38FF-44A6-ABD9-2BEEFAD52DF9}">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.06640625" defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="21.46484375" style="1" customWidth="1"/>
@@ -961,7 +946,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="5" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -983,10 +968,10 @@
     </row>
     <row r="25" spans="1:5" ht="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="4" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>22</v>
@@ -995,26 +980,26 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:5" ht="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="4" t="s">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="6">
-        <v>20</v>
+        <v>84</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>18</v>
@@ -1023,528 +1008,420 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="5" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="4" t="s">
+    <row r="33" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D42" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C33" s="1" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A48" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A49" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" s="1" t="s">
+      <c r="D53" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A59" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A60" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
+      <c r="A61" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="1" t="s">
+      <c r="C61" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="2" t="s">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A67" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A68" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B68" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C39" s="4" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D69" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A53" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A58" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A66" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A68" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A72" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A73" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A74" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A75" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A76" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A77" s="1" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A70" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B70" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B77" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A80" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A81" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A82" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A83" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D83" s="1" t="s">
+      <c r="C70" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>